<commit_message>
feat: SSM register partition columns + Completed MEL backfill sheet
</commit_message>
<xml_diff>
--- a/tests/fixtures/compiler-cable.xlsx
+++ b/tests/fixtures/compiler-cable.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -439,9 +439,23 @@
         <v>C-9001</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v>MTR-9001</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>B14-AHU-7001</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>8</v>
+      </c>
+      <c r="D3" s="2" t="str">
+        <v>C-9002</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: default suffix identity unification — MEL spelling wins across documents
</commit_message>
<xml_diff>
--- a/tests/fixtures/compiler-cable.xlsx
+++ b/tests/fixtures/compiler-cable.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -453,9 +453,23 @@
         <v>C-9002</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="str">
+        <v>DDC-7301</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>B14-LVS-1234</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <v>9</v>
+      </c>
+      <c r="D4" s="2" t="str">
+        <v>C-9003</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>